<commit_message>
Adapt eval_lib evaluation to local Ollama
</commit_message>
<xml_diff>
--- a/data/evaluation_dataset.xlsx
+++ b/data/evaluation_dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI EVAL_files\ai-agent-real-estate-eval\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565DD423-D459-4F09-B625-CE0B0BA5E9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435BC37B-55EF-4646-AD39-6D3E05FAF224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15960" xr2:uid="{BF369E15-F991-6B4A-BC00-4B14A4CF84E4}"/>
   </bookViews>
@@ -66,15 +66,9 @@
     <t>Покажи квартиры с keyword "pet friendly" и переведи цены в евро.</t>
   </si>
   <si>
-    <t>Извлечь объявления, применить текстовый фильтр pet friendly и затем конвертировать цены в EUR.</t>
-  </si>
-  <si>
     <t>Найди квартиры дешевле 1800 долларов, переведи цены в евро и посчитай статистику.</t>
   </si>
   <si>
-    <t>Извлечь объявления, отфильтровать по максимальной цене 1800 USD, конвертировать результат в EUR и вычислить min, max, avg, median по полученным ценам.</t>
-  </si>
-  <si>
     <t>extract_offers, filter_offers, normalize_offers_currency, compute_stats</t>
   </si>
   <si>
@@ -94,6 +88,19 @@
   </si>
   <si>
     <t>RE-005</t>
+  </si>
+  <si>
+    <t>Применить текстовый фильтр «pet friendly». Если подходящих объявлений
+нет, корректно сообщить об отсутствии результатов и не придумывать
+объявления, цены или ссылки. Если объявления найдены, конвертировать
+их цены в EUR и вывести реальные ссылки.</t>
+  </si>
+  <si>
+    <t>Отфильтровать объявления по цене ниже 1800 USD. Если подходящих
+объявлений нет, корректно сообщить об отсутствии результатов и не
+выводить ссылки, цены или вымышленную статистику. Если объявления
+найдены, конвертировать цены в EUR и показать минимум, максимум,
+среднее и медиану.</t>
   </si>
 </sst>
 </file>
@@ -150,10 +157,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -491,13 +501,15 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="49.75" customWidth="1"/>
+    <col min="2" max="2" width="49.75" customWidth="1"/>
+    <col min="3" max="3" width="67" customWidth="1"/>
+    <col min="4" max="4" width="49.75" customWidth="1"/>
     <col min="5" max="5" width="44.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -511,7 +523,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -525,7 +537,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -539,7 +551,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -551,29 +563,29 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="63" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" t="s">
-        <v>13</v>
+      <c r="C6" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>

</xml_diff>